<commit_message>
feat(F-NAR-019): TREE-COL-014 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-014.xlsx
+++ b/stories/arbres/TREE-COL-014.xlsx
@@ -3871,17 +3871,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Nina attrape le seau, toute seule. Elle verse l'eau sur le sable. Le trou se ferme. Le rouge disparaît. Oh. Le seau était à moi, une minute. Je voulais laver le gant. Nina pose le seau, déçue. Tu peux le prendre comment ? S'il te plaît, le seau. Oui. Pour creuser, pas noyer. Nina pousse le sable, cuillère après cuillère. Le pouce rouge revient, un peu propre.</t>
+          <t>Nina attrape le seau, toute seule. Elle verse l'eau sur le sable. Le trou se ferme. Le rouge disparaît. Oh. Le seau était à moi, une minute. Je voulais laver le gant. Nina pose le seau, déçue. Tu le prends avec moi ? S'il te plaît, le seau. Oui. Pour creuser, pas noyer. Nina pousse le sable, cuillère après cuillère. Le pouce rouge revient, un peu propre.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina attrape le seau, toute seule. Elle verse l'eau sur le sable. Le trou se ferme. Le rouge disparaît. Oh. Le seau était à moi, une minute. Je voulais laver le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;. Nina pose le seau, déçue. Tu peux le prendre comment ? S'il te plaît, le seau. Oui. Pour creuser, pas noyer. Nina pousse le sable, cuillère après cuillère. Le pouce rouge revient, un peu propre.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina attrape le seau, toute seule. Elle verse l'eau sur le sable. Le trou se ferme. Le rouge disparaît. Oh. Le seau était à moi, une minute. Je voulais laver le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;. Nina pose le seau, déçue. Tu le prends avec moi ? S'il te plaît, le seau. Oui. Pour creuser, pas noyer. Nina pousse le sable, cuillère après cuillère. Le pouce rouge revient, un peu propre.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina attrape le seau, toute seule. Elle verse l'eau sur le sable. Le trou se ferme. Le rouge disparaît. Oh. Le seau était à moi, une minute. Je voulais laver le &lt;emphasis&gt;gant&lt;/emphasis&gt;. Nina pose le seau, déçue. Tu peux le prendre comment ? S'il te plaît, le seau. Oui. Pour creuser, pas noyer. Nina pousse le sable, cuillère après cuillère. Le pouce rouge revient, un peu propre.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina attrape le seau, toute seule. Elle verse l'eau sur le sable. Le trou se ferme. Le rouge disparaît. Oh. Le seau était à moi, une minute. Je voulais laver le &lt;emphasis&gt;gant&lt;/emphasis&gt;. Nina pose le seau, déçue. Tu le prends avec moi ? S'il te plaît, le seau. Oui. Pour creuser, pas noyer. Nina pousse le sable, cuillère après cuillère. Le pouce rouge revient, un peu propre.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -4027,7 +4027,7 @@
 maman|Le seau était à moi, une minute.
 enfant-f|Je voulais laver le gant.
 narrateur|Nina pose le seau, déçue.
-papa|Tu peux le prendre comment ?
+papa|Tu le prends avec moi ?
 enfant-f|S'il te plaît, le seau.
 maman|Oui.
 maman|Pour creuser, pas noyer.
@@ -5382,17 +5382,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Nina prend le doudou sur le banc. Elle l'enroule autour du gant sableux. La laine du doudou se remplit de grains. Il est sale ! Ce doudou n'aime pas le sable. Je voulais le gant au chaud. Le doudou, tu le prends comment ? S'il te plaît, un coin. Un coin, oui. Pas tout le doudou. Nina frotte le gant avec le coin. Les grains tombent. Le rouge reparaît.</t>
+          <t>Nina prend le doudou sur le banc. Elle l'enroule autour du gant sableux. La laine du doudou se remplit de grains. Il est sale ! Ce doudou n'aime pas le sable. Je voulais le gant au chaud. Le doudou, tu le prends avec moi ? enfant-f|S'il te plaît, un coin. Un coin, oui. Pas tout le doudou. Nina frotte le gant avec le coin. Les grains tombent. Le rouge reparaît.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina prend le doudou sur le banc. Elle l'enroule autour du &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; sableux. La laine du doudou se remplit de grains. Il est sale ! Ce doudou n'aime pas le sable. Je voulais le gant au chaud. Le doudou, tu le prends comment ? S'il te plaît, un coin. Un coin, oui. Pas tout le doudou. Nina frotte le gant avec le coin. Les grains tombent. Le rouge reparaît.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina prend le doudou sur le banc. Elle l'enroule autour du &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; sableux. La laine du doudou se remplit de grains. Il est sale ! Ce doudou n'aime pas le sable. Je voulais le gant au chaud. Le doudou, tu le prends avec moi ? enfant-f|S'il te plaît, un coin. Un coin, oui. Pas tout le doudou. Nina frotte le gant avec le coin. Les grains tombent. Le rouge reparaît.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina prend le doudou sur le banc. Elle l'enroule autour du &lt;emphasis&gt;gant&lt;/emphasis&gt; sableux. La laine du doudou se remplit de grains. Il est sale ! Ce doudou n'aime pas le sable. Je voulais le gant au chaud. Le doudou, tu le prends comment ? S'il te plaît, un coin. Un coin, oui. Pas tout le doudou. Nina frotte le gant avec le coin. Les grains tombent. Le rouge reparaît.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina prend le doudou sur le banc. Elle l'enroule autour du &lt;emphasis&gt;gant&lt;/emphasis&gt; sableux. La laine du doudou se remplit de grains. Il est sale ! Ce doudou n'aime pas le sable. Je voulais le gant au chaud. Le doudou, tu le prends avec moi ? enfant-f|S'il te plaît, un coin. Un coin, oui. Pas tout le doudou. Nina frotte le gant avec le coin. Les grains tombent. Le rouge reparaît.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5536,8 +5536,8 @@
 enfant-f|Il est sale !
 maman|Ce doudou n'aime pas le sable.
 enfant-f|Je voulais le gant au chaud.
-papa|Le doudou, tu le prends comment ?
-enfant-f|S'il te plaît, un coin.
+papa|Le doudou, tu le prends avec moi ?
+papa|enfant-f|S'il te plaît, un coin.
 maman|Un coin, oui.
 maman|Pas tout le doudou.
 narrateur|Nina frotte le gant avec le coin.
@@ -6887,17 +6887,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Nina grimpe le toboggan à l'envers. Le métal pique ses paumes nues. Le gant rouge a glissé en bas. Je l'attrape ! Son pied pousse le gant, par erreur. Le rouge part dans une flaque de boue. Non ! Maman essuie le cartable, plus loin. Elle n'a pas vu le geste. Ça va, Nina ? Le gant. La boue l'a pris. Nina serre les poings, trop petite. Le métal lui refroidit les genoux. J'arrive. Attends une seconde.</t>
+          <t>Nina grimpe le toboggan à l'envers. Le métal pique ses paumes nues. Le gant rouge a glissé en bas. Je l'attrape ! Son pied pousse le gant, par erreur. Le rouge part dans une flaque de boue. Non ! Maman essuie le cartable, plus loin. Elle n'a pas vu le pied. Ça va, Nina ? Le gant. La boue l'a pris. Nina serre les poings, trop petite. Le métal lui refroidit les genoux. J'arrive. Attends une seconde.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina grimpe le toboggan à l'envers. Le métal pique ses paumes nues. Le &lt;emphasis level="moderate"&gt;gant rouge&lt;/emphasis&gt; a glissé en bas. Je l'attrape ! Son pied pousse le gant, par erreur. Le rouge part dans une flaque de boue. Non ! Maman essuie le cartable, plus loin. Elle n'a pas vu le geste. Ça va, Nina ? Le gant. La boue l'a pris. Nina serre les poings, trop petite. Le métal lui refroidit les genoux. J'arrive. Attends une seconde.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina grimpe le toboggan à l'envers. Le métal pique ses paumes nues. Le &lt;emphasis level="moderate"&gt;gant rouge&lt;/emphasis&gt; a glissé en bas. Je l'attrape ! Son pied pousse le gant, par erreur. Le rouge part dans une flaque de boue. Non ! Maman essuie le cartable, plus loin. Elle n'a pas vu le pied. Ça va, Nina ? Le gant. La boue l'a pris. Nina serre les poings, trop petite. Le métal lui refroidit les genoux. J'arrive. Attends une seconde.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Nina grimpe le toboggan à l'envers. Le métal pique ses paumes nues. Le &lt;emphasis&gt;gant rouge&lt;/emphasis&gt; a glissé en bas. Je l'attrape ! Son pied pousse le gant, par erreur. Le rouge part dans une flaque de boue. Non ! Maman essuie le cartable, plus loin. Elle n'a pas vu le geste. Ça va, Nina ? Le gant. La boue l'a pris. Nina serre les poings, trop petite. Le métal lui refroidit les genoux. J'arrive. Attends une seconde. [pause]</t>
+          <t>Nina grimpe le toboggan à l'envers. Le métal pique ses paumes nues. Le &lt;emphasis&gt;gant rouge&lt;/emphasis&gt; a glissé en bas. Je l'attrape ! Son pied pousse le gant, par erreur. Le rouge part dans une flaque de boue. Non ! Maman essuie le cartable, plus loin. Elle n'a pas vu le pied. Ça va, Nina ? Le gant. La boue l'a pris. Nina serre les poings, trop petite. Le métal lui refroidit les genoux. J'arrive. Attends une seconde. [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -7039,7 +7039,7 @@
 narrateur|Le rouge part dans une flaque de boue.
 enfant-f|Non !
 narrateur|Maman essuie le cartable, plus loin.
-narrateur|Elle n'a pas vu le geste.
+narrateur|Elle n'a pas vu le pied.
 maman|Ça va, Nina ?
 enfant-f|Le gant.
 enfant-f|La boue l'a pris.
@@ -7639,17 +7639,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Nina lance le ballon vers la boue. Le ballon tape le gant, puis s'enfonce. Les deux sont pris ! Le ballon n'était pas à toi, Nina. Je voulais pousser le gant. Nina avance, les pieds qui glissent. Tu peux demander, avant de lancer ? S'il te plaît, le ballon. On le sort ensemble, alors. Papa tire le ballon. Le gant bouge. Un lacet rouge se décolle de la boue.</t>
+          <t>Nina lance le ballon vers la boue. Le ballon tape le gant, puis s'enfonce. Les deux sont pris ! Le ballon n'était pas à toi, Nina. Je voulais pousser le gant. Nina avance, les pieds qui glissent. Le ballon, tu le lances où ? S'il te plaît, le ballon. On le sort ensemble, alors. Papa tire le ballon. Le gant bouge. Un lacet rouge se décolle de la boue.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina lance le ballon vers la boue. Le ballon tape le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;, puis s'enfonce. Les deux sont pris ! Le ballon n'était pas à toi, Nina. Je voulais pousser le gant. Nina avance, les pieds qui glissent. Tu peux demander, avant de lancer ? S'il te plaît, le ballon. On le sort ensemble, alors. Papa tire le ballon. Le gant bouge. Un lacet rouge se décolle de la boue.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina lance le ballon vers la boue. Le ballon tape le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;, puis s'enfonce. Les deux sont pris ! Le ballon n'était pas à toi, Nina. Je voulais pousser le gant. Nina avance, les pieds qui glissent. Le ballon, tu le lances où ? S'il te plaît, le ballon. On le sort ensemble, alors. Papa tire le ballon. Le gant bouge. Un lacet rouge se décolle de la boue.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina lance le ballon vers la boue. Le ballon tape le &lt;emphasis&gt;gant&lt;/emphasis&gt;, puis s'enfonce. Les deux sont pris ! Le ballon n'était pas à toi, Nina. Je voulais pousser le gant. Nina avance, les pieds qui glissent. Tu peux demander, avant de lancer ? S'il te plaît, le ballon. On le sort ensemble, alors. Papa tire le ballon. Le gant bouge. Un lacet rouge se décolle de la boue.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina lance le ballon vers la boue. Le ballon tape le &lt;emphasis&gt;gant&lt;/emphasis&gt;, puis s'enfonce. Les deux sont pris ! Le ballon n'était pas à toi, Nina. Je voulais pousser le gant. Nina avance, les pieds qui glissent. Le ballon, tu le lances où ? S'il te plaît, le ballon. On le sort ensemble, alors. Papa tire le ballon. Le gant bouge. Un lacet rouge se décolle de la boue.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -7793,7 +7793,7 @@
 papa|Le ballon n'était pas à toi, Nina.
 enfant-f|Je voulais pousser le gant.
 narrateur|Nina avance, les pieds qui glissent.
-maman|Tu peux demander, avant de lancer ?
+maman|Le ballon, tu le lances où ?
 enfant-f|S'il te plaît, le ballon.
 papa|On le sort ensemble, alors.
 narrateur|Papa tire le ballon.
@@ -9142,17 +9142,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Nina emporte le seau jusqu'au toboggan. Elle verse. L'eau et la boue se mêlent. Le gant nage, plus loin, plus sale. Reviens ! Ce seau servait à rincer les bottes. Je voulais laver le rouge. On verse où, si on demande ? S'il te plaît, un peu d'eau. Un filet, pas tout le seau. Nina penche, tout doucement. La boue s'ouvre. Le gant reste.</t>
+          <t>Nina emporte le seau jusqu'au toboggan. Elle verse. L'eau et la boue se mêlent. Le gant nage, plus loin, plus sale. Reviens ! Ce seau servait à rincer les bottes. Je voulais laver le rouge. On verse où, cette fois ? S'il te plaît, un peu d'eau. Un filet, pas tout le seau. Nina penche, tout doucement. La boue s'ouvre. Le gant reste.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina emporte le seau jusqu'au toboggan. Elle verse. L'eau et la boue se mêlent. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; nage, plus loin, plus sale. Reviens ! Ce seau servait à rincer les bottes. Je voulais laver le rouge. On verse où, si on demande ? S'il te plaît, un peu d'eau. Un filet, pas tout le seau. Nina penche, tout doucement. La boue s'ouvre. Le gant reste.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina emporte le seau jusqu'au toboggan. Elle verse. L'eau et la boue se mêlent. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; nage, plus loin, plus sale. Reviens ! Ce seau servait à rincer les bottes. Je voulais laver le rouge. On verse où, cette fois ? S'il te plaît, un peu d'eau. Un filet, pas tout le seau. Nina penche, tout doucement. La boue s'ouvre. Le gant reste.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina emporte le seau jusqu'au toboggan. Elle verse. L'eau et la boue se mêlent. Le &lt;emphasis&gt;gant&lt;/emphasis&gt; nage, plus loin, plus sale. Reviens ! Ce seau servait à rincer les bottes. Je voulais laver le rouge. On verse où, si on demande ? S'il te plaît, un peu d'eau. Un filet, pas tout le seau. Nina penche, tout doucement. La boue s'ouvre. Le gant reste.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina emporte le seau jusqu'au toboggan. Elle verse. L'eau et la boue se mêlent. Le &lt;emphasis&gt;gant&lt;/emphasis&gt; nage, plus loin, plus sale. Reviens ! Ce seau servait à rincer les bottes. Je voulais laver le rouge. On verse où, cette fois ? S'il te plaît, un peu d'eau. Un filet, pas tout le seau. Nina penche, tout doucement. La boue s'ouvre. Le gant reste.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9297,7 +9297,7 @@
 enfant-f|Reviens !
 maman|Ce seau servait à rincer les bottes.
 enfant-f|Je voulais laver le rouge.
-papa|On verse où, si on demande ?
+papa|On verse où, cette fois ?
 enfant-f|S'il te plaît, un peu d'eau.
 maman|Un filet, pas tout le seau.
 narrateur|Nina penche, tout doucement.
@@ -10654,17 +10654,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Nina glisse le doudou sur le métal. Elle veut attraper le gant, de loin. Le doudou glisse, trop vite, dans la boue. Non, doudou ! Il n'était pas un filet, ce doudou. J'avais froid aux mains. Tu le prends comment, la prochaine ? S'il te plaît, le doudou. On le tient à deux, alors. Nina tient une oreille. Papa l'autre. Le doudou touche le gant, sans tomber.</t>
+          <t>Nina glisse le doudou sur le métal. Elle veut attraper le gant, de loin. Le doudou glisse, trop vite, dans la boue. Non, doudou ! Il n'était pas un filet, ce doudou. J'avais froid aux mains. Tu le prends avec moi, alors ? S'il te plaît, le doudou. On le tient à deux, alors. Nina tient une oreille. Papa l'autre. Le doudou touche le gant, sans tomber.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina glisse le doudou sur le métal. Elle veut attraper le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;, de loin. Le doudou glisse, trop vite, dans la boue. Non, doudou ! Il n'était pas un filet, ce doudou. J'avais froid aux mains. Tu le prends comment, la prochaine ? S'il te plaît, le doudou. On le tient à deux, alors. Nina tient une oreille. Papa l'autre. Le doudou touche le gant, sans tomber.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina glisse le doudou sur le métal. Elle veut attraper le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;, de loin. Le doudou glisse, trop vite, dans la boue. Non, doudou ! Il n'était pas un filet, ce doudou. J'avais froid aux mains. Tu le prends avec moi, alors ? S'il te plaît, le doudou. On le tient à deux, alors. Nina tient une oreille. Papa l'autre. Le doudou touche le gant, sans tomber.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina glisse le doudou sur le métal. Elle veut attraper le &lt;emphasis&gt;gant&lt;/emphasis&gt;, de loin. Le doudou glisse, trop vite, dans la boue. Non, doudou ! Il n'était pas un filet, ce doudou. J'avais froid aux mains. Tu le prends comment, la prochaine ? S'il te plaît, le doudou. On le tient à deux, alors. Nina tient une oreille. Papa l'autre. Le doudou touche le gant, sans tomber.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina glisse le doudou sur le métal. Elle veut attraper le &lt;emphasis&gt;gant&lt;/emphasis&gt;, de loin. Le doudou glisse, trop vite, dans la boue. Non, doudou ! Il n'était pas un filet, ce doudou. J'avais froid aux mains. Tu le prends avec moi, alors ? S'il te plaît, le doudou. On le tient à deux, alors. Nina tient une oreille. Papa l'autre. Le doudou touche le gant, sans tomber.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10808,7 +10808,7 @@
 enfant-f|Non, doudou !
 papa|Il n'était pas un filet, ce doudou.
 enfant-f|J'avais froid aux mains.
-maman|Tu le prends comment, la prochaine ?
+maman|Tu le prends avec moi, alors ?
 enfant-f|S'il te plaît, le doudou.
 papa|On le tient à deux, alors.
 narrateur|Nina tient une oreille.
@@ -11045,17 +11045,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Nino pose le doudou en haut du toboggan. Il veut le faire glisser, comme un luge. Non, il va dans la boue ! C'est drôle ! S'il te plaît, Nino. On le tient. On ne le lance pas. On le tient. Ils tiennent les deux oreilles. Le doudou touche le gant. Papa le saisit. Vous l'avez gardé, au lieu de le jeter.</t>
+          <t>Nino pose le doudou en haut du toboggan. Il veut le faire glisser, comme une luge. Non, il va dans la boue ! C'est drôle ! S'il te plaît, Nino. On le tient. On ne le lance pas. On le tient. Ils tiennent les deux oreilles. Le doudou touche le gant. Papa le saisit. Vous l'avez gardé, au lieu de le jeter.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino pose le doudou en haut du toboggan. Il veut le faire glisser, comme un luge. Non, il va dans la boue ! C'est drôle ! S'il te plaît, Nino. On le tient. On ne le lance pas. On le tient. Ils tiennent les deux oreilles. Le doudou touche le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;. Papa le saisit. Vous l'avez gardé, au lieu de le jeter.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino pose le doudou en haut du toboggan. Il veut le faire glisser, comme une luge. Non, il va dans la boue ! C'est drôle ! S'il te plaît, Nino. On le tient. On ne le lance pas. On le tient. Ils tiennent les deux oreilles. Le doudou touche le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;. Papa le saisit. Vous l'avez gardé, au lieu de le jeter.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nino pose le doudou en haut du toboggan. Il veut le faire glisser, comme un luge. Non, il va dans la boue ! C'est drôle ! S'il te plaît, Nino. On le tient. On ne le lance pas. On le tient. Ils tiennent les deux oreilles. Le doudou touche le &lt;emphasis&gt;gant&lt;/emphasis&gt;. Papa le saisit. Vous l'avez gardé, au lieu de le jeter. [pause]</t>
+          <t>Nino pose le doudou en haut du toboggan. Il veut le faire glisser, comme une luge. Non, il va dans la boue ! C'est drôle ! S'il te plaît, Nino. On le tient. On ne le lance pas. On le tient. Ils tiennent les deux oreilles. Le doudou touche le &lt;emphasis&gt;gant&lt;/emphasis&gt;. Papa le saisit. Vous l'avez gardé, au lieu de le jeter. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11190,7 +11190,7 @@
       <c r="AW54" t="inlineStr">
         <is>
           <t>narrateur|Nino pose le doudou en haut du toboggan.
-narrateur|Il veut le faire glisser, comme un luge.
+narrateur|Il veut le faire glisser, comme une luge.
 enfant-f|Non, il va dans la boue !
 enfant-m|C'est drôle !
 enfant-f|S'il te plaît, Nino.
@@ -13310,17 +13310,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Nino vise le gant avec le ballon. Nina lève les deux mains. Pas trop fort ! Je touche le rouge ! S'il te plaît, Nino. Tout près, pas un coup. Tout près. Nino pose le ballon contre le barreau. Le gant bascule dans les mains de papa. Le coup est devenu un geste. Merci, Nino.</t>
+          <t>Nino vise le gant avec le ballon. Nina lève les deux mains. Pas trop fort ! Je touche le rouge ! S'il te plaît, Nino. Tout près, pas un coup. Tout près. Nino pose le ballon contre le barreau. Le gant bascule dans les mains de papa. Le ballon a poussé, sans frapper. Merci, Nino.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino vise le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; avec le ballon. Nina lève les deux mains. Pas trop fort ! Je touche le rouge ! S'il te plaît, Nino. Tout près, pas un coup. Tout près. Nino pose le ballon contre le barreau. Le gant bascule dans les mains de papa. Le coup est devenu un geste. Merci, Nino.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino vise le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; avec le ballon. Nina lève les deux mains. Pas trop fort ! Je touche le rouge ! S'il te plaît, Nino. Tout près, pas un coup. Tout près. Nino pose le ballon contre le barreau. Le gant bascule dans les mains de papa. Le ballon a poussé, sans frapper. Merci, Nino.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Nino vise le &lt;emphasis&gt;gant&lt;/emphasis&gt; avec le ballon. Nina lève les deux mains. Pas trop fort ! Je touche le rouge ! S'il te plaît, Nino. Tout près, pas un coup. Tout près. Nino pose le ballon contre le barreau. Le gant bascule dans les mains de papa. Le coup est devenu un geste. Merci, Nino. [pause]</t>
+          <t>Nino vise le &lt;emphasis&gt;gant&lt;/emphasis&gt; avec le ballon. Nina lève les deux mains. Pas trop fort ! Je touche le rouge ! S'il te plaît, Nino. Tout près, pas un coup. Tout près. Nino pose le ballon contre le barreau. Le gant bascule dans les mains de papa. Le ballon a poussé, sans frapper. Merci, Nino. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13463,7 +13463,7 @@
 enfant-m|Tout près.
 narrateur|Nino pose le ballon contre le barreau.
 narrateur|Le gant bascule dans les mains de papa.
-maman|Le coup est devenu un geste.
+maman|Le ballon a poussé, sans frapper.
 enfant-f|Merci, Nino.</t>
         </is>
       </c>
@@ -14428,17 +14428,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Nina pose le seau sous la barrière. Elle monte dessus, sans rien dire. Le seau bascule. Nina recule. Ça bouge ! Ce seau n'est pas un tabouret. Le gant est trop haut. Tu veux de l'aide, comment ? S'il te plaît, tu me portes ? Oui. Les pieds au sol, d'abord. Nina attend. Papa s'accroupit. Le seau reste vide, à sa place.</t>
+          <t>Nina pose le seau sous la barrière. Elle monte dessus, sans rien dire. Le seau bascule. Nina recule. Ça bouge ! Ce seau n'est pas un tabouret. Le gant est trop haut. Tu veux que je t'aide ? S'il te plaît, tu me portes ? Oui. Les pieds au sol, d'abord. Nina attend. Papa s'accroupit. Le seau reste vide, à sa place.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina pose le seau sous la barrière. Elle monte dessus, sans rien dire. Le seau bascule. Nina recule. Ça bouge ! Ce seau n'est pas un tabouret. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; est trop haut. Tu veux de l'aide, comment ? S'il te plaît, tu me portes ? Oui. Les pieds au sol, d'abord. Nina attend. Papa s'accroupit. Le seau reste vide, à sa place.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina pose le seau sous la barrière. Elle monte dessus, sans rien dire. Le seau bascule. Nina recule. Ça bouge ! Ce seau n'est pas un tabouret. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; est trop haut. Tu veux que je t'aide ? S'il te plaît, tu me portes ? Oui. Les pieds au sol, d'abord. Nina attend. Papa s'accroupit. Le seau reste vide, à sa place.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina pose le seau sous la barrière. Elle monte dessus, sans rien dire. Le seau bascule. Nina recule. Ça bouge ! Ce seau n'est pas un tabouret. Le &lt;emphasis&gt;gant&lt;/emphasis&gt; est trop haut. Tu veux de l'aide, comment ? S'il te plaît, tu me portes ? Oui. Les pieds au sol, d'abord. Nina attend. Papa s'accroupit. Le seau reste vide, à sa place.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina pose le seau sous la barrière. Elle monte dessus, sans rien dire. Le seau bascule. Nina recule. Ça bouge ! Ce seau n'est pas un tabouret. Le &lt;emphasis&gt;gant&lt;/emphasis&gt; est trop haut. Tu veux que je t'aide ? S'il te plaît, tu me portes ? Oui. Les pieds au sol, d'abord. Nina attend. Papa s'accroupit. Le seau reste vide, à sa place.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14583,7 +14583,7 @@
 enfant-f|Ça bouge !
 maman|Ce seau n'est pas un tabouret.
 enfant-f|Le gant est trop haut.
-papa|Tu veux de l'aide, comment ?
+papa|Tu veux que je t'aide ?
 enfant-f|S'il te plaît, tu me portes ?
 maman|Oui.
 maman|Les pieds au sol, d'abord.
@@ -14821,17 +14821,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Nino monte sur le seau, à son tour. Le seau penche. Nina recule. Ça va tomber ! Je touche ! S'il te plaît, Nino. Pieds par terre. Papa nous porte. Pieds par terre. Nino descend. Papa s'accroupit. Nina demande, bas, le dernier geste. S'il te plaît, tu l'attrapes ? Voilà. Le gant quitte le barreau, dans sa main.</t>
+          <t>Nino monte sur le seau, à son tour. Le seau penche. Nina recule. Ça va tomber ! Je touche ! S'il te plaît, Nino. Pieds par terre. Papa nous porte. Pieds par terre. Nino descend. Papa s'accroupit. Nina parle, bas, une dernière fois. S'il te plaît, tu l'attrapes ? Voilà. Le gant quitte le barreau, dans sa main.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino monte sur le seau, à son tour. Le seau penche. Nina recule. Ça va tomber ! Je touche ! S'il te plaît, Nino. Pieds par terre. Papa nous porte. Pieds par terre. Nino descend. Papa s'accroupit. Nina demande, bas, le dernier geste. S'il te plaît, tu l'attrapes ? Voilà. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; quitte le barreau, dans sa main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino monte sur le seau, à son tour. Le seau penche. Nina recule. Ça va tomber ! Je touche ! S'il te plaît, Nino. Pieds par terre. Papa nous porte. Pieds par terre. Nino descend. Papa s'accroupit. Nina parle, bas, une dernière fois. S'il te plaît, tu l'attrapes ? Voilà. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; quitte le barreau, dans sa main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Nino monte sur le seau, à son tour. Le seau penche. Nina recule. Ça va tomber ! Je touche ! S'il te plaît, Nino. Pieds par terre. Papa nous porte. Pieds par terre. Nino descend. Papa s'accroupit. Nina demande, bas, le dernier geste. S'il te plaît, tu l'attrapes ? Voilà. Le &lt;emphasis&gt;gant&lt;/emphasis&gt; quitte le barreau, dans sa main. [pause]</t>
+          <t>Nino monte sur le seau, à son tour. Le seau penche. Nina recule. Ça va tomber ! Je touche ! S'il te plaît, Nino. Pieds par terre. Papa nous porte. Pieds par terre. Nino descend. Papa s'accroupit. Nina parle, bas, une dernière fois. S'il te plaît, tu l'attrapes ? Voilà. Le &lt;emphasis&gt;gant&lt;/emphasis&gt; quitte le barreau, dans sa main. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14976,7 +14976,7 @@
 enfant-m|Pieds par terre.
 narrateur|Nino descend.
 narrateur|Papa s'accroupit.
-narrateur|Nina demande, bas, le dernier geste.
+narrateur|Nina parle, bas, une dernière fois.
 enfant-f|S'il te plaît, tu l'attrapes ?
 papa|Voilà.
 narrateur|Le gant quitte le barreau, dans sa main.</t>
@@ -15571,17 +15571,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Raphaël regarde l'eau du seau, comme un miroir. Le gant, là-haut ! Je vois le ciel ! Nina attend qu'il lève les yeux. S'il te plaît, Raphaël. Le seau reste. On demande à papa. D'accord. Ils posent le seau. Papa écoute. S'il te plaît, tu le décroches ? Oui. Le gant descend, un barreau à la fois.</t>
+          <t>Raphaël regarde l'eau du seau, comme un miroir. Le gant, là-haut ! Je vois le ciel ! Nina attend qu'il lève les yeux. S'il te plaît, Raphaël. Le seau reste. On appelle papa. D'accord. Ils posent le seau. Papa écoute. S'il te plaît, tu le décroches ? Oui. Le gant descend, un barreau à la fois.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël regarde l'eau du seau, comme un miroir. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;, là-haut ! Je vois le ciel ! Nina attend qu'il lève les yeux. S'il te plaît, Raphaël. Le seau reste. On demande à papa. D'accord. Ils posent le seau. Papa écoute. S'il te plaît, tu le décroches ? Oui. Le gant descend, un barreau à la fois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël regarde l'eau du seau, comme un miroir. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;, là-haut ! Je vois le ciel ! Nina attend qu'il lève les yeux. S'il te plaît, Raphaël. Le seau reste. On appelle papa. D'accord. Ils posent le seau. Papa écoute. S'il te plaît, tu le décroches ? Oui. Le gant descend, un barreau à la fois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Raphaël regarde l'eau du seau, comme un miroir. Le &lt;emphasis&gt;gant&lt;/emphasis&gt;, là-haut ! Je vois le ciel ! Nina attend qu'il lève les yeux. S'il te plaît, Raphaël. Le seau reste. On demande à papa. D'accord. Ils posent le seau. Papa écoute. S'il te plaît, tu le décroches ? Oui. Le gant descend, un barreau à la fois. [pause]</t>
+          <t>Raphaël regarde l'eau du seau, comme un miroir. Le &lt;emphasis&gt;gant&lt;/emphasis&gt;, là-haut ! Je vois le ciel ! Nina attend qu'il lève les yeux. S'il te plaît, Raphaël. Le seau reste. On appelle papa. D'accord. Ils posent le seau. Papa écoute. S'il te plaît, tu le décroches ? Oui. Le gant descend, un barreau à la fois. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15721,7 +15721,7 @@
 narrateur|Nina attend qu'il lève les yeux.
 enfant-f|S'il te plaît, Raphaël.
 enfant-f|Le seau reste.
-enfant-f|On demande à papa.
+enfant-f|On appelle papa.
 enfant-m|D'accord.
 narrateur|Ils posent le seau.
 narrateur|Papa écoute.
@@ -15945,17 +15945,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Nina jette le doudou vers le barreau. Le doudou s'accroche, à côté du gant. Les deux sont coincés ! Le doudou n'était pas un crochet. Je voulais tirer le rouge. On le décroche comment, alors ? S'il te plaît, tu l'attrapes ? Le doudou d'abord. Puis le gant. Nina attend, les bras le long du corps. Papa décroche l'oreille en peluche. Le gant penche, presque libre.</t>
+          <t>Nina jette le doudou vers le barreau. Le doudou s'accroche, à côté du gant. Les deux sont coincés ! Le doudou n'était pas un crochet. Je voulais tirer le rouge. On le décroche à deux, alors ? enfant-f|S'il te plaît, tu l'attrapes ? Le doudou d'abord. Puis le gant. Nina attend, les bras le long du corps. Papa décroche l'oreille en peluche. Le gant penche, presque libre.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina jette le doudou vers le barreau. Le doudou s'accroche, à côté du &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;. Les deux sont coincés ! Le doudou n'était pas un crochet. Je voulais tirer le rouge. On le décroche comment, alors ? S'il te plaît, tu l'attrapes ? Le doudou d'abord. Puis le gant. Nina attend, les bras le long du corps. Papa décroche l'oreille en peluche. Le gant penche, presque libre.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina jette le doudou vers le barreau. Le doudou s'accroche, à côté du &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;. Les deux sont coincés ! Le doudou n'était pas un crochet. Je voulais tirer le rouge. On le décroche à deux, alors ? enfant-f|S'il te plaît, tu l'attrapes ? Le doudou d'abord. Puis le gant. Nina attend, les bras le long du corps. Papa décroche l'oreille en peluche. Le gant penche, presque libre.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina jette le doudou vers le barreau. Le doudou s'accroche, à côté du &lt;emphasis&gt;gant&lt;/emphasis&gt;. Les deux sont coincés ! Le doudou n'était pas un crochet. Je voulais tirer le rouge. On le décroche comment, alors ? S'il te plaît, tu l'attrapes ? Le doudou d'abord. Puis le gant. Nina attend, les bras le long du corps. Papa décroche l'oreille en peluche. Le gant penche, presque libre.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina jette le doudou vers le barreau. Le doudou s'accroche, à côté du &lt;emphasis&gt;gant&lt;/emphasis&gt;. Les deux sont coincés ! Le doudou n'était pas un crochet. Je voulais tirer le rouge. On le décroche à deux, alors ? enfant-f|S'il te plaît, tu l'attrapes ? Le doudou d'abord. Puis le gant. Nina attend, les bras le long du corps. Papa décroche l'oreille en peluche. Le gant penche, presque libre.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -16098,8 +16098,8 @@
 enfant-f|Les deux sont coincés !
 papa|Le doudou n'était pas un crochet.
 enfant-f|Je voulais tirer le rouge.
-maman|On le décroche comment, alors ?
-enfant-f|S'il te plaît, tu l'attrapes ?
+maman|On le décroche à deux, alors ?
+maman|enfant-f|S'il te plaît, tu l'attrapes ?
 papa|Le doudou d'abord.
 papa|Puis le gant.
 narrateur|Nina attend, les bras le long du corps.
@@ -17451,7 +17451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17564,6 +17564,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>